<commit_message>
atualização (modal que avisa novo estoque)
</commit_message>
<xml_diff>
--- a/dados-catalago-pcm-interno/relatorio.xlsx
+++ b/dados-catalago-pcm-interno/relatorio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amaggicombr-my.sharepoint.com/personal/hiago_andre_amaggi_com_br/Documents/Área de Trabalho/codigos/catalogoPecasPCM/dados-catalago-pcm-interno/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="11_FD86FE4AC4094E4AB971B8A5A011EE841C83CB4A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7582CB10-7780-4BA6-BD4C-BE6677DADB7C}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="11_FD86FE4AC4094E4AB971B8A5A011EE841C83CB4A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6E0419C-BC24-4978-8425-39581DB8E83B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5187" uniqueCount="1621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5186" uniqueCount="1621">
   <si>
     <t>Cen.</t>
   </si>
@@ -5334,8 +5334,8 @@
       <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>11</v>
+      <c r="E2" s="2">
+        <v>50</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>12</v>

</xml_diff>